<commit_message>
validación de datos usando bucle de while_true y pedir_numero
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,6 +518,22 @@
         <v>670</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Controles</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D7" t="n">
+        <v>489</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
agregar validacion de datos e IDs dinamicos para excel
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,6 +534,22 @@
         <v>489</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cargador</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>34</v>
+      </c>
+      <c r="D8" t="n">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
agregar busqueda, borrado y re-indexacion automatica de IDs
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -524,14 +524,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Controles</t>
+          <t>Cargador</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>34</v>
       </c>
       <c r="D7" t="n">
-        <v>489</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
@@ -540,14 +540,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cargador</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>